<commit_message>
Reject multi-column merges on the leaf header row for schema.
Propagate horizontal group-row labels into header_name paths, treat 2-row-bidirectional-merge as a schema error, and align horizontal-merge table_schema goldens.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/schema_header_2row/2-row-bidirectional-merge/workbook.xlsx
+++ b/excel/testdata/schema_header_2row/2-row-bidirectional-merge/workbook.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>headerA</t>
   </si>
@@ -32,6 +32,15 @@
   </si>
   <si>
     <t>r5cA</t>
+  </si>
+  <si>
+    <t>r3cB</t>
+  </si>
+  <si>
+    <t>r4cB</t>
+  </si>
+  <si>
+    <t>r5cB</t>
   </si>
   <si>
     <t>r3cC</t>
@@ -364,24 +373,33 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
         <v>5</v>
       </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>